<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-04 Le moulinet de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-04.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché puis jardin</t>
+          <t>marché puis jardin, stand des ailes, table de bois, miel, moulinet, farine, pain, ficelle, vent</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, papa</t>
+          <t>Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut le cerf-volant bleu. Il n'y en a plus. Elle dit qu'elle est déçue. Elle choisit un moulinet. Plus tard, plus de farine. Elle propose des tartines au miel.</t>
+          <t>Les pièces cliquettent. Le sac de pain craque. Sur le bois, un éclat de ficelle luit. Mila veut le cerf-volant bleu, maintenant. Plus d'aile. Épaules basses. Sourire parti. Papa s'accroupit. Je suis déçue. Un moulinet jaune. Merci vécu. Deuxième ruse : plus de farine au jardin. Elle refuse de foncer. Tartines au miel. Un éclat de ficelle tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La toile jaune d'un stand claque. Elle fait un bruit de voile. Des pots de miel brillent au soleil. Le miel est épais et doré. Une abeille marche sur une caisse. La caisse sent le bois chaud. Papa tient un tout petit pot. Tu veux goûter, Mila ? Oui, papa. Mila pose un doigt. Le miel est collant et doux. La place sent le pain chaud. En ce moment, Mila tient la main de papa. Ils marchent entre les stands. Un dessin bleu danse au vent. C'est un cerf-volant, tout haut. Celui-là, papa. Le bleu. On va demander. Le stand est presque vide. Il reste des ficelles, pas d'aile. Il n'y en a plus, Mila. Mila sent ses épaules tomber. Sa gorge se serre un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Mila souffle une fois. L'air du marché lui chatouille le nez. Un moulinet jaune tourne sur une table. Ses pales font un petit cliquetis. Celui-là, alors. Une autre idée. Bravo, Mila. Papa prend le moulinet. Mila le fait tourner. Le jaune virevolte contre le ciel. Plus tard, ils rentrent au jardin. La table de bois est tiède. Le moulinet tourne encore, tout seul. On fait un gâteau au miel ? Je regarde la farine. Papa ouvre le placard. Le sachet est plat, tout vide. Il n'y a plus de farine. Mila sent encore ses épaules tomber. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Mila regarde le petit pot. Des tartines au miel, alors. Oui. Tu as proposé autre chose. Ils tartinent ensemble. Le miel file, lent et collant. Le pain sent le chaud. C'est sucré. Au marché, puis ici, c'est pareil. On nomme : déçue. Puis on cherche une autre idée. Le moulinet tourne sur la table. Une miette reste collée au doigt de Mila.</t>
+          <t>Les pièces de papa cliquettent dans sa paume. Ça fait tic, papa. Tu entends les pièces, Mila ? Oui, papa. Le sac de pain de maman craque contre la joue. Il est chaud, maman. Tu le sens, le pain ? Oui, il sent le chaud. Le vent du marché tire une ficelle blanche. Elle danse, maman. Elle tape le clou, tu vois ? Oui, un petit tic. Sur le bois, un éclat de ficelle luit. Il brille, papa. Le soleil le touche. Un point clair. Des pots de miel attendent, collants et lourds. Ça sent le sucré. Tu veux un doigt de miel ? Un tout petit, maman. Mila pose un doigt sur le pot ouvert. Le miel file, lent, sur la peau. Il colle. Il est épais, oui. Une pale de papier tremble, loin, au-dessus. C'est bleu, papa. Tu le vois, là-haut ? Oui, ça danse. En ce moment, Mila cherche le bleu du ciel. Le cerf-volant, maintenant ! Celui qui danse, là-haut ? Oui, le bleu, papa. Ils marchent vers le stand des ailes. Je le prends, maman. On va demander, Mila ? Oui, tout de suite. Le stand est presque vide, sous le vent. Il reste des ficelles, pas d'aile bleue. Il n'y en a plus, Mila. Plus de bleu ? Mila reste surprise, les mains ouvertes. Ses épaules tombent d'un coup. Sa gorge se serre, près du stand. Oh. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Tu as les épaules basses, Mila ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Mila ? Un peu, maman. Je suis déçue. Un moulinet jaune tourne sur la table. Ses pales font un petit cliquetis. Celui-là, alors. L'éclat de ficelle tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La toile jaune d'un stand claque. Elle fait un bruit de voile. Des pots de miel brillent au soleil. Le miel est épais et doré. Une abeille marche sur une caisse. La caisse sent le bois chaud. Papa tient un tout petit pot. Tu veux goûter, Mila ? Oui, papa. Mila pose un doigt. Le miel est collant et doux. La place sent le pain chaud. En ce moment, Mila tient la main de papa. Ils marchent entre les stands. Un dessin bleu danse au vent. C'est un cerf-volant, tout haut. Celui-là, papa. Le bleu. On va demander. Le stand est presque vide. Il reste des ficelles, pas d'aile. Il n'y en a plus, Mila. Mila sent ses épaules tomber. Sa gorge se serre un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Mila souffle une fois. L'air du marché lui chatouille le nez. Un moulinet jaune tourne sur une table. Ses pales font un petit cliquetis. Celui-là, alors. Une autre idée. Bravo, Mila. Papa prend le moulinet. Mila le fait tourner. Le jaune virevolte contre le ciel. Plus tard, ils rentrent au jardin. La table de bois est tiède. Le moulinet tourne encore, tout seul. On fait un gâteau au miel ? Je regarde la farine. Papa ouvre le placard. Le sachet est plat, tout vide. Il n'y a plus de farine. Mila sent encore ses épaules tomber. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Mila regarde le petit pot. Des tartines au miel, alors. Oui. Tu as proposé autre chose. Ils tartinent ensemble. Le miel file, lent et collant. Le pain sent le chaud. C'est sucré. Au marché, puis ici, c'est pareil. On nomme : déçue. Puis on cherche une autre idée. Le moulinet tourne sur la table. Une miette reste collée au doigt de Mila.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les pièces de papa cliquettent dans sa paume. Ça fait tic, papa. Tu entends les pièces, Mila ? Oui, papa. Le sac de pain de maman craque contre la joue. Il est chaud, maman. Tu le sens, le pain ? Oui, il sent le chaud. Le vent du marché tire une ficelle blanche. Elle danse, maman. Elle tape le clou, tu vois ? Oui, un petit tic. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de ficelle&lt;/emphasis&gt; luit. Il brille, papa. Le soleil le touche. Un point clair. Des pots de miel attendent, collants et lourds. Ça sent le sucré. Tu veux un doigt de miel ? Un tout petit, maman. Mila pose un doigt sur le pot ouvert. Le miel file, lent, sur la peau. Il colle. Il est épais, oui. Une pale de papier tremble, loin, au-dessus. C'est bleu, papa. Tu le vois, là-haut ? Oui, ça danse. En ce moment, Mila cherche le bleu du ciel. Le cerf-volant, maintenant ! Celui qui danse, là-haut ? Oui, le bleu, papa. Ils marchent vers le stand des ailes. Je le prends, maman. On va demander, Mila ? Oui, tout de suite. Le stand est presque vide, sous le vent. Il reste des ficelles, pas d'aile bleue. Il n'y en a plus, Mila. Plus de bleu ? Mila reste surprise, les mains ouvertes. Ses épaules tombent d'un coup. Sa gorge se serre, près du stand. Oh. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Tu as les épaules basses, Mila ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Mila ? Un peu, maman. Je suis déçue. Un moulinet jaune tourne sur la table. Ses pales font un petit cliquetis. Celui-là, alors. L'éclat de ficelle tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Cléa marche au marché. Sa main est dans la main de papa. Elle sent l'odeur du miel. Elle veut un cerf-volant bleu. Le marchand dit : il n'y en a plus. Cléa sent ses épaules tomber. Sa gorge se serre. Cléa dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Être déçu, ce n'est pas honteux. Papa s'accroupit. Papa dit : un souhait peut attendre. On peut chercher une autre idée. Cléa souffle une fois. Elle regarde un moulinet jaune. Elle dit : celui-là, alors. Papa sourit. Ils achètent le moulinet. Cléa le fait tourner. Plus tard, ils rentrent au jardin. Cléa veut faire un gâteau au miel. Papa ouvre le placard. Il n'y a plus de farine. Cléa sent encore les épaules tomber. Elle dit : je suis déçue. Papa dit : une autre idée. Cléa propose des tartines au miel. Papa dit : oui. Elles tartinent ensemble. Le miel est collant. Au marché, puis au jardin, c'est pareil. On nomme : déçu. Puis on cherche une autre idée. [pause]</t>
+          <t>Les pièces de papa cliquettent dans sa paume. Ça fait tic, papa. Tu entends les pièces, Mila ? Oui, papa. Le sac de pain de maman craque contre la joue. Il est chaud, maman. Tu le sens, le pain ? Oui, il sent le chaud. Le vent du marché tire une ficelle blanche. Elle danse, maman. Elle tape le clou, tu vois ? Oui, un petit tic. Sur le bois, un &lt;emphasis&gt;éclat de ficelle&lt;/emphasis&gt; luit. Il brille, papa. Le soleil le touche. Un point clair. Des pots de miel attendent, collants et lourds. Ça sent le sucré. Tu veux un doigt de miel ? Un tout petit, maman. Mila pose un doigt sur le pot ouvert. Le miel file, lent, sur la peau. Il colle. Il est épais, oui. Une pale de papier tremble, loin, au-dessus. C'est bleu, papa. Tu le vois, là-haut ? Oui, ça danse. En ce moment, Mila cherche le bleu du ciel. Le cerf-volant, maintenant ! Celui qui danse, là-haut ? Oui, le bleu, papa. Ils marchent vers le stand des ailes. Je le prends, maman. On va demander, Mila ? Oui, tout de suite. Le stand est presque vide, sous le vent. Il reste des ficelles, pas d'aile bleue. Il n'y en a plus, Mila. Plus de bleu ? Mila reste surprise, les mains ouvertes. Ses épaules tombent d'un coup. Sa gorge se serre, près du stand. Oh. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Tu as les épaules basses, Mila ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Mila ? Un peu, maman. Je suis déçue. Un moulinet jaune tourne sur la table. Ses pales font un petit cliquetis. Celui-là, alors. L'éclat de ficelle tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de ficelle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,73 +1321,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_cerf_volant_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La toile jaune d'un stand claque.
-narrateur|Elle fait un bruit de voile.
-narrateur|Des pots de miel brillent au soleil.
-narrateur|Le miel est épais et doré.
-narrateur|Une abeille marche sur une caisse.
-narrateur|La caisse sent le bois chaud.
-narrateur|Papa tient un tout petit pot.
-papa|Tu veux goûter, Mila ?
+          <t>narrateur|Les pièces de papa cliquettent dans sa paume.
+enfant-f|Ça fait tic, papa.
+papa|Tu entends les pièces, Mila ?
 enfant-f|Oui, papa.
-narrateur|Mila pose un doigt.
-narrateur|Le miel est collant et doux.
-narrateur|La place sent le pain chaud.
-narrateur|En ce moment, Mila tient la main de papa.
-narrateur|Ils marchent entre les stands.
-narrateur|Un dessin bleu danse au vent.
-narrateur|C'est un cerf-volant, tout haut.
-enfant-f|Celui-là, papa.
-enfant-f|Le bleu.
-papa|On va demander.
-narrateur|Le stand est presque vide.
-narrateur|Il reste des ficelles, pas d'aile.
+narrateur|Le sac de pain de maman craque contre la joue.
+enfant-f|Il est chaud, maman.
+maman|Tu le sens, le pain ?
+enfant-f|Oui, il sent le chaud.
+narrateur|Le vent du marché tire une ficelle blanche.
+enfant-f|Elle danse, maman.
+maman|Elle tape le clou, tu vois ?
+enfant-f|Oui, un petit tic.
+narrateur|Sur le bois, un éclat de ficelle luit.
+enfant-f|Il brille, papa.
+papa|Le soleil le touche.
+enfant-f|Un point clair.
+narrateur|Des pots de miel attendent, collants et lourds.
+enfant-f|Ça sent le sucré.
+maman|Tu veux un doigt de miel ?
+enfant-f|Un tout petit, maman.
+narrateur|Mila pose un doigt sur le pot ouvert.
+narrateur|Le miel file, lent, sur la peau.
+enfant-f|Il colle.
+papa|Il est épais, oui.
+narrateur|Une pale de papier tremble, loin, au-dessus.
+enfant-f|C'est bleu, papa.
+papa|Tu le vois, là-haut ?
+enfant-f|Oui, ça danse.
+narrateur|En ce moment, Mila cherche le bleu du ciel.
+enfant-f|Le cerf-volant, maintenant !
+papa|Celui qui danse, là-haut ?
+enfant-f|Oui, le bleu, papa.
+narrateur|Ils marchent vers le stand des ailes.
+enfant-f|Je le prends, maman.
+maman|On va demander, Mila ?
+enfant-f|Oui, tout de suite.
+narrateur|Le stand est presque vide, sous le vent.
+narrateur|Il reste des ficelles, pas d'aile bleue.
 papa|Il n'y en a plus, Mila.
-narrateur|Mila sent ses épaules tomber.
-narrateur|Sa gorge se serre un peu.
+enfant-f|Plus de bleu ?
+narrateur|Mila reste surprise, les mains ouvertes.
+narrateur|Ses épaules tombent d'un coup.
+narrateur|Sa gorge se serre, près du stand.
+enfant-f|Oh.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+papa|Tu as les épaules basses, Mila ?
+enfant-f|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Mila ?
+enfant-f|Un peu, maman.
 enfant-f|Je suis déçue.
-papa|Tu es déçue.
-papa|Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On peut chercher une autre idée.
-narrateur|Mila souffle une fois.
-narrateur|L'air du marché lui chatouille le nez.
-narrateur|Un moulinet jaune tourne sur une table.
+narrateur|Un moulinet jaune tourne sur la table.
 narrateur|Ses pales font un petit cliquetis.
 enfant-f|Celui-là, alors.
-papa|Une autre idée.
-papa|Bravo, Mila.
-narrateur|Papa prend le moulinet.
-narrateur|Mila le fait tourner.
-narrateur|Le jaune virevolte contre le ciel.
-narrateur|Plus tard, ils rentrent au jardin.
-narrateur|La table de bois est tiède.
-narrateur|Le moulinet tourne encore, tout seul.
-enfant-f|On fait un gâteau au miel ?
-papa|Je regarde la farine.
-narrateur|Papa ouvre le placard.
-narrateur|Le sachet est plat, tout vide.
-papa|Il n'y a plus de farine.
-narrateur|Mila sent encore ses épaules tomber.
-enfant-f|Je suis déçue.
-papa|Encore un souhait qui attend.
-papa|Une autre idée ?
-narrateur|Mila regarde le petit pot.
-enfant-f|Des tartines au miel, alors.
-papa|Oui.
-papa|Tu as proposé autre chose.
-narrateur|Ils tartinent ensemble.
-narrateur|Le miel file, lent et collant.
-narrateur|Le pain sent le chaud.
-enfant-f|C'est sucré.
-papa|Au marché, puis ici, c'est pareil.
-papa|On nomme : déçue.
-papa|Puis on cherche une autre idée.
-narrateur|Le moulinet tourne sur la table.
-narrateur|Une miette reste collée au doigt de Mila.</t>
+narrateur|L'éclat de ficelle tremble, puis tient.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>marche,vent</t>
         </is>
       </c>
     </row>
@@ -1419,12 +1421,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le cerf-volant n'est plus là. Que dit Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le cerf-volant n'est plus là. Que dit &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le cerf-volant n'est plus là. Que dit Cléa ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le cerf-volant n'est plus là. Que dit &lt;emphasis&gt;Mila&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1449,7 +1451,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Cléa cherche une autre idée. Que dit-elle d'abord ?</t>
+          <t>Mila cherche une autre idée. Que dit-elle d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1487,18 +1489,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1513,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1549,23 +1555,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_cerf_volant_n_est_plus_la_que_dit_mila; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1598,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a encore du miel au doigt. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Bravo, Mila. Le moulinet, puis les tartines. Deux autres idées. Oui. Le pain est encore un peu chaud.</t>
+          <t>Mila reste près du stand, un moment. Le bleu n'est plus là. Les mots se bousculent dans sa bouche. Je veux le jaune, alors. Mila avance la main, trop vite. Puis elle s'arrête. Elle referme la bouche, près des pales. Personne ne parle, sous le vent. Elle observe le moulinet, un instant. Il tourne, papa. Tu le prends, Mila ? Oui, une autre idée. Merci, Mila. Papa reste à la même hauteur. Les pales sont jaunes, Mila ? Oui, maman. Papa donne une pièce au stand. Le moulinet passe dans la main de Mila. Il est léger. Tu le sens, le vent ? Oui, papa. On rentre au jardin, Mila ? Oui, avec le jaune. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On marche, sans se presser ? Oui. Le sac de pain tape la hanche de maman. Le pain est chaud. Il sent le four, Mila ? Oui, maman. Le jaune tourne contre le ciel ? Oui, papa. Une pale cliquette contre le pouce. Ça chatouille.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a encore du miel au doigt. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Bravo, Mila. Le moulinet, puis les tartines. Deux autres idées. Oui. Le pain est encore un peu chaud.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila reste près du stand, un moment. Le bleu n'est plus là. Les mots se bousculent dans sa bouche. Je veux le jaune, alors. Mila avance la main, trop vite. Puis elle s'arrête. Elle referme la bouche, près des pales. Personne ne parle, sous le vent. Elle observe le &lt;emphasis level="moderate"&gt;moulinet&lt;/emphasis&gt;, un instant. Il tourne, papa. Tu le prends, Mila ? Oui, une autre idée. Merci, Mila. Papa reste à la même hauteur. Les pales sont jaunes, Mila ? Oui, maman. Papa donne une pièce au stand. Le moulinet passe dans la main de Mila. Il est léger. Tu le sens, le vent ? Oui, papa. On rentre au jardin, Mila ? Oui, avec le jaune. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On marche, sans se presser ? Oui. Le sac de pain tape la hanche de maman. Le pain est chaud. Il sent le four, Mila ? Oui, maman. Le jaune tourne contre le ciel ? Oui, papa. Une pale cliquette contre le pouce. Ça chatouille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Cléa a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Le souhait peut attendre. Une autre idée est arrivée. [pause]</t>
+          <t>Mila reste près du stand, un moment. Le bleu n'est plus là. Les mots se bousculent dans sa bouche. Je veux le jaune, alors. Mila avance la main, trop vite. Puis elle s'arrête. Elle referme la bouche, près des pales. Personne ne parle, sous le vent. Elle observe le &lt;emphasis&gt;moulinet&lt;/emphasis&gt;, un instant. Il tourne, papa. Tu le prends, Mila ? Oui, une autre idée. Merci, Mila. Papa reste à la même hauteur. Les pales sont jaunes, Mila ? Oui, maman. Papa donne une pièce au stand. Le moulinet passe dans la main de Mila. Il est léger. Tu le sens, le vent ? Oui, papa. On rentre au jardin, Mila ? Oui, avec le jaune. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On marche, sans se presser ? Oui. Le sac de pain tape la hanche de maman. Le pain est chaud. Il sent le four, Mila ? Oui, maman. Le jaune tourne contre le ciel ? Oui, papa. Une pale cliquette contre le pouce. Ça chatouille. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1655,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1663,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1689,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>moulinet</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1721,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1737,21 +1743,51 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_l_autre_idée; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_prend_le_moulinet_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a encore du miel au doigt.
-enfant-f|J'ai dit : je suis déçue.
-papa|Oui.
-papa|Le souhait peut attendre.
-papa|Une autre idée est arrivée.
-papa|Bravo, Mila.
-papa|Le moulinet, puis les tartines.
-enfant-f|Deux autres idées.
-papa|Oui.
-narrateur|Le pain est encore un peu chaud.</t>
+          <t>narrateur|Mila reste près du stand, un moment.
+enfant-f|Le bleu n'est plus là.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Je veux le jaune, alors.
+narrateur|Mila avance la main, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Elle referme la bouche, près des pales.
+narrateur|Personne ne parle, sous le vent.
+narrateur|Elle observe le moulinet, un instant.
+enfant-f|Il tourne, papa.
+papa|Tu le prends, Mila ?
+enfant-f|Oui, une autre idée.
+papa|Merci, Mila.
+narrateur|Papa reste à la même hauteur.
+maman|Les pales sont jaunes, Mila ?
+enfant-f|Oui, maman.
+narrateur|Papa donne une pièce au stand.
+narrateur|Le moulinet passe dans la main de Mila.
+enfant-f|Il est léger.
+papa|Tu le sens, le vent ?
+enfant-f|Oui, papa.
+maman|On rentre au jardin, Mila ?
+enfant-f|Oui, avec le jaune.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On marche, sans se presser ?
+enfant-f|Oui.
+narrateur|Le sac de pain tape la hanche de maman.
+enfant-f|Le pain est chaud.
+maman|Il sent le four, Mila ?
+enfant-f|Oui, maman.
+papa|Le jaune tourne contre le ciel ?
+enfant-f|Oui, papa.
+narrateur|Une pale cliquette contre le pouce.
+enfant-f|Ça chatouille.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>moulinet</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1814,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila croque la tartine. Le miel lui colle aux lèvres. On reste un peu au jardin ? Oui, papa. Tu as nommé : déçue. Puis tu as cherché. Le moulinet tourne sur la table. Une abeille passe, loin, et s'en va. Le miel est bon. Et l'autre idée aussi.</t>
+          <t>Au jardin, la table de bois est tiède. Le gâteau au miel, maintenant ! Mila court vers le placard, trop vite. La farine, papa ! Je l'ouvre, le placard. Papa ouvre le placard, près de l'eau. Le sachet de farine est plat, vide. Il n'y a plus de farine. Plus de gâteau ? Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. J'attends. Personne ne dit la suite. Elle observe le moulinet, un instant. Elle écoute le jardin, près de la table. Sur le bois, un éclat de ficelle luit. Là, sur le bois. Tu vois le point, Mila ? Oui, papa. La ficelle du moulinet brille au soleil. C'est la même, maman. Tu la reconnais ? Oui, du marché. Mila regarde le pot de miel. Des tartines, alors. Le pain du sac, Mila ? Oui, maman. On tartine, sans se presser ? Oui, papa. Maman pose le pain sur le bois. Le miel file, lent, sur la tartine. Il colle aux doigts. Il est sucré, Mila ? Oui, maman. Le jaune tourne près du pot ? Oui, tout près. Une miette reste collée au pouce de Mila. Elle est sucrée.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila croque la tartine. Le miel lui colle aux lèvres. On reste un peu au jardin ? Oui, papa. Tu as nommé : déçue. Puis tu as cherché. Le moulinet tourne sur la table. Une abeille passe, loin, et s'en va. Le miel est bon. Et l'autre idée aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au jardin, la table de bois est tiède. Le gâteau au miel, maintenant ! Mila court vers le placard, trop vite. La farine, papa ! Je l'ouvre, le placard. Papa ouvre le placard, près de l'eau. Le sachet de farine est plat, vide. Il n'y a plus de farine. Plus de gâteau ? Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. J'attends. Personne ne dit la suite. Elle observe le moulinet, un instant. Elle écoute le jardin, près de la table. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de ficelle&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Mila ? Oui, papa. La ficelle du moulinet brille au soleil. C'est la même, maman. Tu la reconnais ? Oui, du marché. Mila regarde le pot de miel. Des tartines, alors. Le pain du sac, Mila ? Oui, maman. On tartine, sans se presser ? Oui, papa. Maman pose le pain sur le bois. Le miel file, lent, sur la tartine. Il colle aux doigts. Il est sucré, Mila ? Oui, maman. Le jaune tourne près du pot ? Oui, tout près. Une miette reste collée au pouce de Mila. Elle est sucrée.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Cléa croque la tartine. Le moulinet tourne sur la table. [pause]</t>
+          <t>Au jardin, la table de bois est tiède. Le gâteau au miel, maintenant ! Mila court vers le placard, trop vite. La farine, papa ! Je l'ouvre, le placard. Papa ouvre le placard, près de l'eau. Le sachet de farine est plat, vide. Il n'y a plus de farine. Plus de gâteau ? Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. J'attends. Personne ne dit la suite. Elle observe le moulinet, un instant. Elle écoute le jardin, près de la table. Sur le bois, un &lt;emphasis&gt;éclat de ficelle&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Mila ? Oui, papa. La ficelle du moulinet brille au soleil. C'est la même, maman. Tu la reconnais ? Oui, du marché. Mila regarde le pot de miel. Des tartines, alors. Le pain du sac, Mila ? Oui, maman. On tartine, sans se presser ? Oui, papa. Maman pose le pain sur le bois. Le miel file, lent, sur la tartine. Il colle aux doigts. Il est sucré, Mila ? Oui, maman. Le jaune tourne près du pot ? Oui, tout près. Une miette reste collée au pouce de Mila. Elle est sucrée. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,7 +1871,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1843,10 +1879,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1903,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de ficelle</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1937,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1911,19 +1951,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=plus_de_farine_elle_refuse_de_foncer_tartines; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila croque la tartine.
-narrateur|Le miel lui colle aux lèvres.
-papa|On reste un peu au jardin ?
+          <t>narrateur|Au jardin, la table de bois est tiède.
+enfant-f|Le gâteau au miel, maintenant !
+narrateur|Mila court vers le placard, trop vite.
+enfant-f|La farine, papa !
+papa|Je l'ouvre, le placard.
+narrateur|Papa ouvre le placard, près de l'eau.
+narrateur|Le sachet de farine est plat, vide.
+papa|Il n'y a plus de farine.
+enfant-f|Plus de gâteau ?
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+enfant-f|J'attends.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le moulinet, un instant.
+narrateur|Elle écoute le jardin, près de la table.
+narrateur|Sur le bois, un éclat de ficelle luit.
+enfant-f|Là, sur le bois.
+papa|Tu vois le point, Mila ?
 enfant-f|Oui, papa.
-papa|Tu as nommé : déçue.
-papa|Puis tu as cherché.
-narrateur|Le moulinet tourne sur la table.
-narrateur|Une abeille passe, loin, et s'en va.
-enfant-f|Le miel est bon.
-papa|Et l'autre idée aussi.</t>
+narrateur|La ficelle du moulinet brille au soleil.
+enfant-f|C'est la même, maman.
+maman|Tu la reconnais ?
+enfant-f|Oui, du marché.
+narrateur|Mila regarde le pot de miel.
+enfant-f|Des tartines, alors.
+maman|Le pain du sac, Mila ?
+enfant-f|Oui, maman.
+papa|On tartine, sans se presser ?
+enfant-f|Oui, papa.
+narrateur|Maman pose le pain sur le bois.
+narrateur|Le miel file, lent, sur la tartine.
+enfant-f|Il colle aux doigts.
+maman|Il est sucré, Mila ?
+enfant-f|Oui, maman.
+papa|Le jaune tourne près du pot ?
+enfant-f|Oui, tout près.
+narrateur|Une miette reste collée au pouce de Mila.
+enfant-f|Elle est sucrée.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>placard</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2029,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Mila. Le moulinet s'arrête, tout doux.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de miel. Le bleu n'était plus là, papa. Tu l'as vu, toi ? Oui, près du stand. On est bien, ici. Mila tapote une pale du doigt. Elle a une trace de miel. Tu la vois, la trace ? Oui, maman. Le moulinet est resté, Mila. Oui, avec le jaune. Ça sent le pain, un peu tiède. Et le miel, maman. Oui, dans l'air. Le jardin est doux, Mila ? Oui, papa. Le moulinet reste près du pot. Il tourne, tout seul. On laisse le jaune, Mila ? Oui, tout près. Un éclat de ficelle tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Mila. Le moulinet s'arrête, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de miel. Le bleu n'était plus là, papa. Tu l'as vu, toi ? Oui, près du stand. On est bien, ici. Mila tapote une pale du doigt. Elle a une trace de miel. Tu la vois, la trace ? Oui, maman. Le moulinet est resté, Mila. Oui, avec le jaune. Ça sent le pain, un peu tiède. Et le miel, maman. Oui, dans l'air. Le jardin est doux, Mila ? Oui, papa. Le moulinet reste près du pot. Il tourne, tout seul. On laisse le jaune, Mila ? Oui, tout près. Un &lt;emphasis level="moderate"&gt;éclat de ficelle&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de miel. Le bleu n'était plus là, papa. Tu l'as vu, toi ? Oui, près du stand. On est bien, ici. Mila tapote une pale du doigt. Elle a une trace de miel. Tu la vois, la trace ? Oui, maman. Le moulinet est resté, Mila. Oui, avec le jaune. Ça sent le pain, un peu tiède. Et le miel, maman. Oui, dans l'air. Le jardin est doux, Mila ? Oui, papa. Le moulinet reste près du pot. Il tourne, tout seul. On laisse le jaune, Mila ? Oui, tout près. Un &lt;emphasis&gt;éclat de ficelle&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,18 +2086,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2106,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2120,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de ficelle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2143,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,27 +2156,54 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-papa|Bravo, Mila.
-narrateur|Le moulinet s'arrête, tout doux.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de miel.
+enfant-f|Le bleu n'était plus là, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près du stand.
+maman|On est bien, ici.
+narrateur|Mila tapote une pale du doigt.
+enfant-f|Elle a une trace de miel.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le moulinet est resté, Mila.
+enfant-f|Oui, avec le jaune.
+narrateur|Ça sent le pain, un peu tiède.
+enfant-f|Et le miel, maman.
+maman|Oui, dans l'air.
+papa|Le jardin est doux, Mila ?
+enfant-f|Oui, papa.
+narrateur|Le moulinet reste près du pot.
+enfant-f|Il tourne, tout seul.
+papa|On laisse le jaune, Mila ?
+enfant-f|Oui, tout près.
+narrateur|Un éclat de ficelle tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>moulinet</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2164,6 +2274,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>